<commit_message>
git add backtest/engine.py backtest/strategy.py backtest/costs.py git commit -m "Add SMA strategy, cost model + weight guard"
</commit_message>
<xml_diff>
--- a/output/screener_results.xlsx
+++ b/output/screener_results.xlsx
@@ -834,7 +834,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:H18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -844,6 +844,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -896,6 +897,11 @@
           <t>net_debt_ebitda</t>
         </is>
       </c>
+      <c r="H3" s="17" t="inlineStr">
+        <is>
+          <t>n_factors</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
@@ -904,16 +910,16 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>83.09999999999999</v>
+        <v>82.7</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>90.23</v>
+        <v>93.67</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>62.94</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="F4" s="18" t="n">
         <v>0</v>
@@ -921,6 +927,9 @@
       <c r="G4" s="18" t="n">
         <v>2.93</v>
       </c>
+      <c r="H4" s="18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -929,72 +938,81 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>75.2</v>
+        <v>80</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>80.61</v>
+        <v>47.44</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>4.77</v>
+        <v>12.35</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="F5" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="20" t="n">
-        <v>5.87</v>
+        <v>5.77</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>MGRC</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>60.7</v>
+          <t>PRGS</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>68.2</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>13.78</v>
+        <v>16.96</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>40.71</v>
+        <v>5.77</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>0.01</v>
       </c>
       <c r="G6" s="18" t="n">
-        <v>1.55</v>
+        <v>4.15</v>
+      </c>
+      <c r="H6" s="18" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
         <is>
-          <t>EPAC</t>
+          <t>MGRC</t>
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>55.5</v>
+        <v>57.1</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>14.69</v>
+        <v>13.83</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>20.08</v>
+        <v>41.13</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>0.61</v>
+        <v>1.55</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1004,16 +1022,16 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>54.4</v>
+        <v>51.6</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>13.68</v>
+        <v>11.53</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>9.869999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>0.16</v>
+        <v>0.09</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>0.02</v>
@@ -1021,30 +1039,36 @@
       <c r="G8" s="18" t="n">
         <v>2.65</v>
       </c>
+      <c r="H8" s="18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>EPAC</t>
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>53.8</v>
+        <v>50.1</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>16.52</v>
+        <v>14.51</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>5.2</v>
+        <v>20.12</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>0.29</v>
+        <v>0.21</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>4.15</v>
+        <v>0.61</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1054,16 +1078,16 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>53.1</v>
+        <v>49.6</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>13.16</v>
+        <v>12.34</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>17.59</v>
+        <v>16.78</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>0</v>
@@ -1071,55 +1095,62 @@
       <c r="G10" s="18" t="n">
         <v>0.23</v>
       </c>
+      <c r="H10" s="18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>SKYW</t>
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>52</v>
+        <v>48.8</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>20.43</v>
-      </c>
-      <c r="D11" s="20" t="n">
-        <v>11.03</v>
-      </c>
+        <v>8.19</v>
+      </c>
+      <c r="D11" s="20" t="inlineStr"/>
       <c r="E11" s="20" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="G11" s="20" t="n">
-        <v>-1.9</v>
+        <v>1.79</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>UFPI</t>
-        </is>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>45.5</v>
+          <t>HCSG</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>38.7</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>10.9</v>
+        <v>19.76</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>16.98</v>
+        <v>11.04</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>0.01</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-1.9</v>
+      </c>
+      <c r="H12" s="18" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1129,16 +1160,16 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>32.9</v>
+        <v>36.2</v>
       </c>
       <c r="C13" s="20" t="n">
-        <v>12.89</v>
+        <v>13.6</v>
       </c>
       <c r="D13" s="20" t="n">
-        <v>18.98</v>
+        <v>20.3</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>0.41</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F13" s="20" t="n">
         <v>0.01</v>
@@ -1146,70 +1177,84 @@
       <c r="G13" s="20" t="n">
         <v>-0.98</v>
       </c>
+      <c r="H13" s="20" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="18" t="inlineStr">
         <is>
-          <t>CALM</t>
+          <t>UFPI</t>
         </is>
       </c>
       <c r="B14" s="22" t="n">
-        <v>21.7</v>
+        <v>35.9</v>
       </c>
       <c r="C14" s="18" t="n">
-        <v>1.53</v>
+        <v>10.93</v>
       </c>
       <c r="D14" s="18" t="n">
-        <v>3.36</v>
+        <v>17.28</v>
       </c>
       <c r="E14" s="18" t="n">
-        <v>0.47</v>
+        <v>0.12</v>
       </c>
       <c r="F14" s="18" t="n">
-        <v>0.12</v>
+        <v>0.01</v>
       </c>
       <c r="G14" s="18" t="n">
-        <v>-0.68</v>
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="H14" s="18" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="20" t="inlineStr">
         <is>
-          <t>HTLD</t>
-        </is>
-      </c>
-      <c r="B15" s="20" t="inlineStr"/>
-      <c r="C15" s="20" t="inlineStr"/>
-      <c r="D15" s="20" t="inlineStr"/>
-      <c r="E15" s="20" t="n">
-        <v>-0.06</v>
-      </c>
+          <t>CALM</t>
+        </is>
+      </c>
+      <c r="B15" s="22" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="C15" s="20" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="D15" s="20" t="n">
+        <v>3.48</v>
+      </c>
+      <c r="E15" s="20" t="inlineStr"/>
       <c r="F15" s="20" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="G15" s="20" t="n">
-        <v>1.06</v>
+        <v>-0.68</v>
+      </c>
+      <c r="H15" s="20" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="18" t="inlineStr">
         <is>
-          <t>SKYW</t>
+          <t>HTLD</t>
         </is>
       </c>
       <c r="B16" s="18" t="inlineStr"/>
-      <c r="C16" s="18" t="n">
-        <v>7.98</v>
-      </c>
+      <c r="C16" s="18" t="inlineStr"/>
       <c r="D16" s="18" t="inlineStr"/>
       <c r="E16" s="18" t="n">
-        <v>0.18</v>
+        <v>-0.05</v>
       </c>
       <c r="F16" s="18" t="n">
         <v>0.05</v>
       </c>
       <c r="G16" s="18" t="n">
-        <v>1.79</v>
+        <v>1.06</v>
+      </c>
+      <c r="H16" s="18" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17">
@@ -1221,11 +1266,14 @@
       <c r="B17" s="20" t="inlineStr"/>
       <c r="C17" s="20" t="inlineStr"/>
       <c r="D17" s="20" t="n">
-        <v>10.69</v>
+        <v>11.45</v>
       </c>
       <c r="E17" s="20" t="inlineStr"/>
       <c r="F17" s="20" t="inlineStr"/>
       <c r="G17" s="20" t="inlineStr"/>
+      <c r="H17" s="20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
@@ -1236,16 +1284,19 @@
       <c r="B18" s="18" t="inlineStr"/>
       <c r="C18" s="18" t="inlineStr"/>
       <c r="D18" s="18" t="n">
-        <v>8.210000000000001</v>
+        <v>8.869999999999999</v>
       </c>
       <c r="E18" s="18" t="inlineStr"/>
       <c r="F18" s="18" t="inlineStr"/>
       <c r="G18" s="18" t="inlineStr"/>
+      <c r="H18" s="18" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1257,7 +1308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1267,6 +1318,7 @@
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1319,6 +1371,11 @@
           <t>net_debt_ebitda</t>
         </is>
       </c>
+      <c r="H3" s="17" t="inlineStr">
+        <is>
+          <t>n_factors</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="18" t="inlineStr">
@@ -1327,16 +1384,16 @@
         </is>
       </c>
       <c r="B4" s="19" t="n">
-        <v>83.09999999999999</v>
+        <v>82.7</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>90.23</v>
+        <v>93.67</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>62.94</v>
+        <v>67.65000000000001</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="F4" s="18" t="n">
         <v>0</v>
@@ -1344,6 +1401,9 @@
       <c r="G4" s="18" t="n">
         <v>2.93</v>
       </c>
+      <c r="H4" s="18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="20" t="inlineStr">
@@ -1352,72 +1412,81 @@
         </is>
       </c>
       <c r="B5" s="19" t="n">
-        <v>75.2</v>
+        <v>80</v>
       </c>
       <c r="C5" s="20" t="n">
-        <v>80.61</v>
+        <v>47.44</v>
       </c>
       <c r="D5" s="20" t="n">
-        <v>4.77</v>
+        <v>12.35</v>
       </c>
       <c r="E5" s="20" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="F5" s="20" t="n">
         <v>0</v>
       </c>
       <c r="G5" s="20" t="n">
-        <v>5.87</v>
+        <v>5.77</v>
+      </c>
+      <c r="H5" s="20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="18" t="inlineStr">
         <is>
-          <t>MGRC</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="n">
-        <v>60.7</v>
+          <t>PRGS</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="n">
+        <v>68.2</v>
       </c>
       <c r="C6" s="18" t="n">
-        <v>13.78</v>
+        <v>16.96</v>
       </c>
       <c r="D6" s="18" t="n">
-        <v>40.71</v>
+        <v>5.77</v>
       </c>
       <c r="E6" s="18" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="F6" s="18" t="n">
         <v>0.01</v>
       </c>
       <c r="G6" s="18" t="n">
-        <v>1.55</v>
+        <v>4.15</v>
+      </c>
+      <c r="H6" s="18" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="20" t="inlineStr">
         <is>
-          <t>EPAC</t>
+          <t>MGRC</t>
         </is>
       </c>
       <c r="B7" s="21" t="n">
-        <v>55.5</v>
+        <v>57.1</v>
       </c>
       <c r="C7" s="20" t="n">
-        <v>14.69</v>
+        <v>13.83</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>20.08</v>
+        <v>41.13</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="F7" s="20" t="n">
-        <v>0.02</v>
+        <v>0.01</v>
       </c>
       <c r="G7" s="20" t="n">
-        <v>0.61</v>
+        <v>1.55</v>
+      </c>
+      <c r="H7" s="20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1427,16 +1496,16 @@
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>54.4</v>
+        <v>51.6</v>
       </c>
       <c r="C8" s="18" t="n">
-        <v>13.68</v>
+        <v>11.53</v>
       </c>
       <c r="D8" s="18" t="n">
-        <v>9.869999999999999</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="E8" s="18" t="n">
-        <v>0.16</v>
+        <v>0.09</v>
       </c>
       <c r="F8" s="18" t="n">
         <v>0.02</v>
@@ -1444,30 +1513,36 @@
       <c r="G8" s="18" t="n">
         <v>2.65</v>
       </c>
+      <c r="H8" s="18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="20" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>EPAC</t>
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>53.8</v>
+        <v>50.1</v>
       </c>
       <c r="C9" s="20" t="n">
-        <v>16.52</v>
+        <v>14.51</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>5.2</v>
+        <v>20.12</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>0.29</v>
+        <v>0.21</v>
       </c>
       <c r="F9" s="20" t="n">
-        <v>0.01</v>
+        <v>0.02</v>
       </c>
       <c r="G9" s="20" t="n">
-        <v>4.15</v>
+        <v>0.61</v>
+      </c>
+      <c r="H9" s="20" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1477,16 +1552,16 @@
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>53.1</v>
+        <v>49.6</v>
       </c>
       <c r="C10" s="18" t="n">
-        <v>13.16</v>
+        <v>12.34</v>
       </c>
       <c r="D10" s="18" t="n">
-        <v>17.59</v>
+        <v>16.78</v>
       </c>
       <c r="E10" s="18" t="n">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="F10" s="18" t="n">
         <v>0</v>
@@ -1494,55 +1569,62 @@
       <c r="G10" s="18" t="n">
         <v>0.23</v>
       </c>
+      <c r="H10" s="18" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="20" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>SKYW</t>
         </is>
       </c>
       <c r="B11" s="21" t="n">
-        <v>52</v>
+        <v>48.8</v>
       </c>
       <c r="C11" s="20" t="n">
-        <v>20.43</v>
-      </c>
-      <c r="D11" s="20" t="n">
-        <v>11.03</v>
-      </c>
+        <v>8.19</v>
+      </c>
+      <c r="D11" s="20" t="inlineStr"/>
       <c r="E11" s="20" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="F11" s="20" t="n">
-        <v>0.01</v>
+        <v>0.05</v>
       </c>
       <c r="G11" s="20" t="n">
-        <v>-1.9</v>
+        <v>1.79</v>
+      </c>
+      <c r="H11" s="20" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="18" t="inlineStr">
         <is>
-          <t>UFPI</t>
-        </is>
-      </c>
-      <c r="B12" s="21" t="n">
-        <v>45.5</v>
+          <t>HCSG</t>
+        </is>
+      </c>
+      <c r="B12" s="22" t="n">
+        <v>38.7</v>
       </c>
       <c r="C12" s="18" t="n">
-        <v>10.9</v>
+        <v>19.76</v>
       </c>
       <c r="D12" s="18" t="n">
-        <v>16.98</v>
+        <v>11.04</v>
       </c>
       <c r="E12" s="18" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="F12" s="18" t="n">
         <v>0.01</v>
       </c>
       <c r="G12" s="18" t="n">
-        <v>-0.6899999999999999</v>
+        <v>-1.9</v>
+      </c>
+      <c r="H12" s="18" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -1552,16 +1634,16 @@
         </is>
       </c>
       <c r="B13" s="22" t="n">
-        <v>32.9</v>
+        <v>36.2</v>
       </c>
       <c r="C13" s="20" t="n">
-        <v>12.89</v>
+        <v>13.6</v>
       </c>
       <c r="D13" s="20" t="n">
-        <v>18.98</v>
+        <v>20.3</v>
       </c>
       <c r="E13" s="20" t="n">
-        <v>0.41</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="F13" s="20" t="n">
         <v>0.01</v>
@@ -1569,11 +1651,14 @@
       <c r="G13" s="20" t="n">
         <v>-0.98</v>
       </c>
+      <c r="H13" s="20" t="n">
+        <v>5</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>